<commit_message>
Ajuste nos path e correcao do path do campo buscar
</commit_message>
<xml_diff>
--- a/app/saida/resultado_busca_maps.xlsx
+++ b/app/saida/resultado_busca_maps.xlsx
@@ -481,12 +481,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4,3</t>
+          <t>4,2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>800</t>
+          <t>812</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>216</t>
+          <t>217</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -644,13 +644,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="93" customWidth="1" min="4" max="4"/>
+    <col width="117" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="64" customWidth="1" min="6" max="6"/>
   </cols>
@@ -700,7 +700,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>275</t>
+          <t>284</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>542</t>
+          <t>549</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -754,103 +754,103 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BlueFit Biagi</t>
+          <t>Allp Fit Ribeirão Preto</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4,3</t>
+          <t>4,5</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>336</t>
+          <t>33</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Av. Maurílio Biagi, 1450 - Santa Cruz do Jose Jacques, Ribeirão Preto - SP, 14020-750</t>
+          <t>Av. Dr. Francisco Junqueira, 2534 - Vila Seixas, Ribeirão Preto - SP, 14020-000</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>(16) 99738-7868</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.bluefit.com.br/unidade/biagi</t>
+          <t>https://allpfit.com.br/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Academia Gaviões 24h - Ribeirão Preto</t>
+          <t>Academia BlueFit Biagi</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4,1</t>
+          <t>4,4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>348</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Av. Dom Pedro I, 1200 - Ipiranga, Ribeirão Preto - SP, 14055-630</t>
+          <t>Av. Maurílio Biagi, 1450 - Santa Cruz do Jose Jacques, Ribeirão Preto - SP, 14020-750</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>(11) 94074-7584</t>
+          <t>Não encontrado</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://academiagavioes.com.br/unidades/item/spribeiraopreto</t>
+          <t>https://www.bluefit.com.br/unidade/biagi</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RP Fitness Academia | Lutas e Musculação | Ribeirão Preto</t>
+          <t>Academia Gaviões 24h - Ribeirão Preto</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4,7</t>
+          <t>4,2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>217</t>
+          <t>309</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>R. Guarujá, 27 - Jardim Paulista, Ribeirão Preto - SP, 14090-102</t>
+          <t>Av. Dom Pedro I, 1200 - Ipiranga, Ribeirão Preto - SP, 14055-630</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>(16) 98189-3355</t>
+          <t>(11) 94074-7584</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://rpfitness.com.br/links</t>
+          <t>https://academiagavioes.com.br/unidades/item/spribeiraopreto</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Boa Forma Fitness - Academia</t>
+          <t>Prime Academia Ribeirão Preto</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -860,54 +860,54 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>293</t>
+          <t>129</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>R. André Rebouças, 739 - Ipiranga, Ribeirão Preto - SP, 14055-650</t>
+          <t>Alameda Domingos F. Vilas Bôas, 946 - Parque dos Lagos, Ribeirão Preto - SP, 14094-164</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>(16) 99212-1774</t>
+          <t>(16) 99427-4085</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/boaformafitnessrp/</t>
+          <t>https://www.instagram.com/primeacademiarp?igsh=eDd0ZnM5N3N1bWd4</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Prime Academia Ribeirão Preto</t>
+          <t>RP Fitness Academia | Lutas e Musculação | Ribeirão Preto</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4,9</t>
+          <t>4,7</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>217</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Alameda Domingos F. Vilas Bôas, 946 - Parque dos Lagos, Ribeirão Preto - SP, 14094-164</t>
+          <t>R. Guarujá, 27 - Jardim Paulista, Ribeirão Preto - SP, 14090-102</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>(16) 99427-4085</t>
+          <t>(16) 98189-3355</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/primeacademiarp?igsh=eDd0ZnM5N3N1bWd4</t>
+          <t>https://rpfitness.com.br/links</t>
         </is>
       </c>
     </row>
@@ -924,7 +924,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>115</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>473</t>
+          <t>476</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -978,32 +978,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MB Fit Academia</t>
+          <t>Boa Forma Fitness - Academia</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4,7</t>
+          <t>4,9</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>296</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Av. José Herbert Faleiros, 510 - Recreio das Acacias, Ribeirão Preto - SP, 14098-780</t>
+          <t>R. André Rebouças, 739 - Ipiranga, Ribeirão Preto - SP, 14055-650</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>(16) 3235-2902</t>
+          <t>(16) 99212-1774</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/mb_fit_academia/</t>
+          <t>https://www.instagram.com/boaformafitnessrp/</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>143</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>322</t>
+          <t>323</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1074,59 +1074,59 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BlueFit Nova Aliança</t>
+          <t>Platz Academia</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>4,1</t>
+          <t>4,9</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>378</t>
+          <t>66</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Av. Dr. José Cesário Monteiro da Silva, 385 - Nova Aliança, Ribeirão Preto - SP, 14026-600</t>
+          <t>Avenida Antônio Machado Santa'Anna, 50 - City Ribeirão, Ribeirão Preto - SP, 14021-230</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>(16) 99604-7245</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.bluefit.com.br/unidade/nova-alianca</t>
+          <t>Não disponível</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Skyfit - Unidade Ribeirão Preto</t>
+          <t>Academia Pulsar Ribeirão Preto</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>4,2</t>
+          <t>4,7</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>32</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>R. Silveira Martins, 774 - Campos Elísios, Ribeirão Preto - SP, 14080-625</t>
+          <t>R. Valentim Mestriner, 475 - Iguatemi, Ribeirão Preto - SP, 14091-420</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>(16) 99963-7999</t>
+          <t>(16) 3618-1050</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1148,22 +1148,182 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
+          <t>123</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>R. Franco da Rocha, 1370 - Vila Virginia, Ribeirão Preto - SP, 14030-356</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>(16) 99223-8286</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://bit.ly/Academiagoogle</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Academia BlueFit Nova Aliança</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>4,1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Av. Dr. José Cesário Monteiro da Silva, 385 - Nova Aliança, Ribeirão Preto - SP, 14026-600</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Não encontrado</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://www.bluefit.com.br/unidade/nova-alianca</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ForBody Academia - Unidade 1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>4,7</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
           <t>106</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>R. Franco da Rocha, 1370 - Vila Virginia, Ribeirão Preto - SP, 14030-356</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>(16) 99223-8286</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>https://bit.ly/Academiagoogle</t>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>R. Triunfo, 385 - Santa Cruz do Jose Jacques, Ribeirão Preto - SP, 14020-670</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>(16) 99437-4366</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>http://www.forbodyacademia.com.br/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Academia Universal</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>4,8</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>171</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>R. Ten. Catão Roxo, 1612 - Jardim Antartica, Ribeirão Preto - SP, 14051-140</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>(16) 99796-4682</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>http://www.academiauniversalrp.com.br/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Power House Fitness Gym</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>5,0</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>R. Dr. Jorge Lobato, 678 - Vila Tiberio, Ribeirão Preto - SP, 14050-110</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Não encontrado</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://instagram.com/powerhouse.fitnessgym</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Companhia Athletica Ribeirão Preto</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>4,7</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Avenida Coronel Fernando Ferreira Leite, 1540 RibeirãoShopping - Jardim Nova Alianca, Ribeirão Preto - SP, 14026-900</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>(16) 3917-5000</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>http://ciaathletica.com.br/ribeirao-shopping/</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -1186,7 +1346,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="92" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="89" customWidth="1" min="6" max="6"/>
+    <col width="75" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1224,32 +1384,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Evino Moema</t>
+          <t>Cortés Asador Villa-Lobos</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4,9</t>
+          <t>4,3</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>954</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Av. Pavão, 683 - Recanto Paraíso, São Paulo - SP, 04516-012</t>
+          <t>Av. das Nações Unidas, 4777 - Jardim Universidade Pinheiros, São Paulo - SP, 05477-000</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>(11) 97626-7350</t>
+          <t>(11) 3474-6030</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Não disponível</t>
+          <t>https://restaurantecortes.com.br/</t>
         </is>
       </c>
     </row>
@@ -1261,12 +1421,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>4,9</t>
+          <t>4,8</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>140</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1298,7 +1458,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>35.095</t>
+          <t>36.524</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1330,7 +1490,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>14.553</t>
+          <t>14.801</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1345,7 +1505,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://acasadoporco.com.br/o-restaurante/</t>
+          <t>https://reservation-widget.tagme.com.br/smartlink/616efc96ffe80e0011e599d8</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1522,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.326</t>
+          <t>5.348</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1384,39 +1544,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Parrillada Fuego Celeste - Unidade Moema</t>
+          <t>L'Osteria do Piero</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>4,8</t>
+          <t>4,6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2.099</t>
+          <t>2.471</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Av. Jacutinga, 365 - Indianópolis, São Paulo - SP, 04515-030</t>
+          <t>Alameda Franca, 1509 - Cerqueira César, São Paulo - SP, 01422-001</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>(11) 5051-7575</t>
+          <t>(11) 3086-1010</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/fuegocelesteoficial/?hl=pt-br</t>
+          <t>http://www.losteriadopiero.com.br/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Parrillada Fuego Celeste - Unidade Vila Mariana</t>
+          <t>Parrillada Fuego Celeste - Unidade Moema</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1426,17 +1586,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4.031</t>
+          <t>2.287</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>R. Joaquim Távora, 1068 - Vila Mariana, São Paulo - SP, 04015-012</t>
+          <t>Av. Jacutinga, 365 - Indianópolis, São Paulo - SP, 04515-030</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>(11) 4563-8999</t>
+          <t>(11) 5051-7575</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1448,135 +1608,135 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>D.O.M.</t>
+          <t>Restaurante Porque Sim</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4,6</t>
+          <t>4,7</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2.627</t>
+          <t>6.448</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>R. Barão de Capanema, 549 - Jardins, São Paulo - SP, 01411-010</t>
+          <t>R. Thomaz Gonzaga, 75 - Liberdade, São Paulo - SP, 01506-020</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>(11) 96918-9947</t>
+          <t>(11) 3277-1557</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>http://domrestaurante.com.br/</t>
+          <t>https://www.instagram.com/restauranteporquesim/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Adega Santiago Asador</t>
+          <t>Esther Rooftop</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>4,7</t>
+          <t>4,5</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>3.659</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Rua Haddock Lobo, 1626 - Cerqueira César, São Paulo - SP, 01414-002</t>
+          <t>01045-000, R. Basílio da Gama, 29 - Conjunto 1101 - República, São Paulo - SP, 01046-020</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>(11) 3198-8258</t>
+          <t>(11) 3256-1009</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>http://www.adegasantiago.com.br/</t>
+          <t>https://www.estherrooftop.com.br/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Zucco Ristorante: Cozinha Italiana, Contemporâneo, Risotos, Massas, Vinhos SP</t>
+          <t>Sapori d'Italia Limeira Cucina &amp; Bar</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4,8</t>
+          <t>4,7</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3.745</t>
+          <t>410</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Rua Haddock Lobo, 1416 - Cerqueira César, São Paulo - SP, 01414-002</t>
+          <t>Rua São Vicente de Paulo, 423 - São Cristovam, Limeira - SP, 13480-590</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>(11) 3897-0666</t>
+          <t>(19) 3702-2031</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://ristorante.zucco.com.br/</t>
+          <t>http://www.saporilimeira.com.br/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Restaurante Expresso São Paulo</t>
+          <t>Parrillada Fuego Celeste - Unidade Vila Mariana</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4,4</t>
+          <t>4,8</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>894</t>
+          <t>4.078</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>R. da Quitanda, 123 - Centro Histórico de São Paulo, São Paulo - SP, 01012-010</t>
+          <t>R. Joaquim Távora, 1068 - Vila Mariana, São Paulo - SP, 04015-012</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>(11) 99487-8931</t>
+          <t>(11) 4563-8999</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/expressosaopaulo/</t>
+          <t>https://www.instagram.com/fuegocelesteoficial/?hl=pt-br</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Coco Bambu</t>
+          <t>Coco Bambu - SP Market</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1586,7 +1746,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23.816</t>
+          <t>24.392</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1608,71 +1768,71 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>HUB Food Art Lounge</t>
+          <t>Zucco Ristorante: Cozinha Italiana, Contemporâneo, Risotos, Massas, Vinhos SP</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>4,6</t>
+          <t>4,8</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>605</t>
+          <t>4.294</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>R. Olimpíadas, 205 - Vila Olímpia, São Paulo - SP, 04551-000</t>
+          <t>Rua Haddock Lobo, 1416 - Cerqueira César, São Paulo - SP, 01414-002</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>(11) 3049-6689</t>
+          <t>(11) 3897-0666</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.hubrestaurante.com/?utm_source=Referral&amp;utm_medium=AccorHotels</t>
+          <t>https://ristorante.zucco.com.br/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>L'Osteria do Piero</t>
+          <t>Restaurante Expresso São Paulo</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>4,6</t>
+          <t>4,4</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2.441</t>
+          <t>895</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Alameda Franca, 1509 - Cerqueira César, São Paulo - SP, 01422-001</t>
+          <t>R. da Quitanda, 123 - Centro Histórico de São Paulo, São Paulo - SP, 01012-010</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>(11) 3086-1010</t>
+          <t>(11) 99487-8931</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>http://www.losteriadopiero.com.br/</t>
+          <t>https://www.instagram.com/expressosaopaulo/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TastelT Restaurante</t>
+          <t>HUB Food Art Lounge</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1682,182 +1842,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>808</t>
+          <t>610</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Rua Joinville, 515 - Vila Mariana, São Paulo - SP, 04008-001</t>
+          <t>R. Olimpíadas, 205 - Vila Olímpia, São Paulo - SP, 04551-000</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>(11) 5088-4000</t>
+          <t>(11) 3049-6689</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>http://tasteitrestaurante.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Restaurante Sapporo</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>4,8</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>5.336</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Praça Nossa Sra. Aparecida, 114 - Moema, São Paulo - SP, 04075-010</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>(11) 5054-5140</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>http://www.restaurantesapporo.com.br/</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Tatini Restaurante</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>4,7</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>2.023</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>R. Batataes, 558 - Jardim Paulista, São Paulo - SP, 01423-010</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>(11) 3885-7601</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>http://restaurantetatini.com.br/</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Restaurante Porque Sim</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>4,7</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>6.390</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>R. Thomaz Gonzaga, 75 - Liberdade, São Paulo - SP, 01506-020</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>(11) 3277-1557</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/restauranteporquesim/</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>CIPÓRESTÔ</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>4,8</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>309</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>R. Olimpíadas, 205 - Vila Olímpia, São Paulo - SP, 04551-000</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>(11) 3049-6622</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>https://restaurants.accorhotels.com/pt-br/restaurant-8942_R001-ciporesto-sao-paulo.shtml</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Vicolo Nostro</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>4,7</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>4.926</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Rua Jataituba, 29 - Cidade Monções, São Paulo - SP, 04704-090</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>(11) 5561-5287</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>https://vicolonostro.com.br/</t>
+          <t>https://www.hubrestaurante.com/?utm_source=Referral&amp;utm_medium=AccorHotels</t>
         </is>
       </c>
     </row>
@@ -1872,15 +1872,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="51" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="109" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="77" customWidth="1" min="6" max="6"/>
+    <col width="57" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1918,155 +1918,155 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Dra Flavia Machado - Reumatologia, Piracicaba - SP</t>
+          <t>Dr Fábio do Carmo Duarte Geriatra em Piracicaba</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4,7</t>
+          <t>4,9</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>53</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>R. Samuel Neves, 635 - Jardim Europa, Piracicaba - SP, 13416-404</t>
+          <t>R. do Vergueiro, 409 - Centro, Piracicaba - SP, 13400-770</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>(19) 98413-5202</t>
+          <t>(19) 98408-2706</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://flaviareumatologista.com.br/</t>
+          <t>https://drfabioduartegeriatra.com.br/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dentista 24hrs Piracicaba - Pitta Odontologia</t>
+          <t>Clínica da Cidade - Piracicaba</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>4,6</t>
+          <t>4,7</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>882</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Av. Barão de Serra Negra, 886 - Vila Rezende, Piracicaba - SP, 13405-220</t>
+          <t>Av. Independência, 1075 - Alto, Piracicaba - SP, 13419-155</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>(19) 99960-9427</t>
+          <t>(19) 3052-7627</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/clinica24horaspiracicaba?igsh=MW1vOG81eDlhcTJ0cw==</t>
+          <t>https://clinicadacidade.com.br/centro-medico/piracicaba/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Clínica da Cidade - Piracicaba</t>
+          <t>Clínica Bom Jesus</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4,7</t>
+          <t>3,4</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>830</t>
+          <t>91</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Av. Independência, 1075 - Alto, Piracicaba - SP, 13419-155</t>
+          <t>R. José Pinto de Almeida, 788 - Centro, Piracicaba - SP, 13419-000</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>(19) 3052-7627</t>
+          <t>(19) 3302-9754</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://clinicadacidade.com.br/centro-medico/piracicaba/</t>
+          <t>http://clinimedpiracicaba.com.br/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Clínica Bom Jesus</t>
+          <t>Centermed Clínica</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3,0</t>
+          <t>3,9</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>51</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>R. José Pinto de Almeida, 788 - Centro, Piracicaba - SP, 13419-000</t>
+          <t>R. Praça José Bonifácio, 839 - Centro, Piracicaba - SP, 13400-340</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>(19) 3302-9754</t>
+          <t>(19) 3927-5600</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>http://clinimedpiracicaba.com.br/</t>
+          <t>http://www.centermedclinica.com.br/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Centro Clínico Paulista</t>
+          <t>Clínica Piracicaba Privamed</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3,7</t>
+          <t>4,8</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>50</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Av. Dr. Edgar Conceição, 779 - sala 9 - Paulista, Piracicaba - SP, 13401-100</t>
+          <t>R. Espírito Santo, 179 - Piracicamirim, Piracicaba - SP, 13420-505</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>(19) 3422-0948</t>
+          <t>(19) 3432-1112</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2078,320 +2078,160 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Centermed Clínica</t>
+          <t>Clinica Moraes</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>3,9</t>
+          <t>4,6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>780</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>R. Praça José Bonifácio, 839 - Centro, Piracicaba - SP, 13400-340</t>
+          <t>Condomínio Edifício Primus Center - Av. Independência, 350 - SALA 161/162 - Alto, Piracicaba - SP, 13419-160</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>(19) 3927-5600</t>
+          <t>(19) 3374-6209</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>http://www.centermedclinica.com.br/</t>
+          <t>http://www.clinicamoraes.com.br/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Clínica Saúde Integrada Piracicaba</t>
+          <t>Centro Clínico Paulista</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4,7</t>
+          <t>3,5</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Av. Independência, 3053 - Alemães, Piracicaba - SP, 13416-240</t>
+          <t>Av. Dr. Edgar Conceição, 779 - sala 9 - Paulista, Piracicaba - SP, 13401-100</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>(19) 97146-5713</t>
+          <t>(19) 3422-0948</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://csipiracicaba.com.br/</t>
+          <t>Não disponível</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Clínica Piracicaba Privamed</t>
+          <t>Clínica Bragalha</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4,8</t>
+          <t>4,2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>110</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Av. Dona Jane Conceição, 1181 - Jaraguá, Piracicaba - SP, 13403-030</t>
+          <t>R. Gomes Carneiro, 1729 - Alto, Piracicaba - SP, 13419-165</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>(19) 3432-1112</t>
+          <t>(19) 3402-4008</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Não disponível</t>
+          <t>http://www.clinicabragalha.com.br/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Clinica Moraes</t>
+          <t>Clínica Saúde Integrada Piracicaba</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>4,5</t>
+          <t>3,9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>698</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Condomínio Edifício Primus Center - Av. Independência, 350 - SALA 161/162 - Alto, Piracicaba - SP, 13419-160</t>
+          <t>Av. Independência, 3053 - Alemães, Piracicaba - SP, 13416-240</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>(19) 3374-6209</t>
+          <t>(19) 97146-5713</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>http://www.clinicamoraes.com.br/</t>
+          <t>https://csipiracicaba.com.br/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Clínica Bragalha</t>
+          <t>Up Clin Clínica de Especialidades</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>4,3</t>
+          <t>4,7</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>14</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>R. Gomes Carneiro, 1729 - Alto, Piracicaba - SP, 13419-165</t>
+          <t>Av. Independência, 699 - Alto, Piracicaba - SP, 13419-155</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>(19) 3402-4008</t>
+          <t>(19) 3402-6513</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>http://www.clinicabragalha.com.br/</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Clínica de Especialidades Piracicaba</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>4,5</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>R. São João, 1202 - Alto, Piracicaba - SP, 13400-390</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>(19) 3422-4270</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Não disponível</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Clínica Médica Divino Dr. Piracicaba</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Não informada</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Não informada</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>R. Dom Pedro II, 936 - Centro, Piracicaba - SP, 13400-390</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>(11) 97607-3356</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>https://divinodoutor.com.br/</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Clínicas LQ - Unidade Piracicaba</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>5,0</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>262</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Av. Dr. Edgar Conceição, 779 - sala 03 - Paulista, Piracicaba - SP, 13401-100</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>(19) 98448-8688</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>https://lq.med.br/</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Up Clin Clínica de Especialidades</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>4,7</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Av. Independência, 699 - Alto, Piracicaba - SP, 13419-155</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>(19) 3402-6513</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
           <t>https://clinicaupclin.com.br/</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>AmorSaúde Piracicaba</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>3,0</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>R. Dom Pedro II, 790 - Centro, Piracicaba - SP, 13400-390</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>(19) 3374-2001</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>https://amorsaude.com.br/</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -2452,32 +2292,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Festval Batel</t>
+          <t>Supermercado Condor Agua Verde</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>4,7</t>
+          <t>4,2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>5.476</t>
+          <t>13.107</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>R. Cel. Dulcídio, 880 - Batel, Curitiba - PR, 80420-170</t>
+          <t>Av. Água Verde, 860 - Água Verde, Curitiba - PR, 80620-200</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>(41) 3014-1590</t>
+          <t>(41) 3888-2229</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://festval.com/</t>
+          <t>https://www.condor.com.br/</t>
         </is>
       </c>
     </row>
@@ -2494,7 +2334,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1.560</t>
+          <t>1.569</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2526,7 +2366,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2.859</t>
+          <t>2.881</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2548,32 +2388,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Supermercado Condor Agua Verde</t>
+          <t>Festval Batel</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4,2</t>
+          <t>4,7</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>13.072</t>
+          <t>5.610</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Av. Água Verde, 860 - Água Verde, Curitiba - PR, 80620-200</t>
+          <t>R. Cel. Dulcídio, 880 - Batel, Curitiba - PR, 80420-170</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>(41) 3888-2229</t>
+          <t>(41) 3014-1590</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.condor.com.br/</t>
+          <t>https://festval.com/</t>
         </is>
       </c>
     </row>
@@ -2590,7 +2430,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14.858</t>
+          <t>14.968</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2606,166 +2446,6 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>https://www.carrefour.com.br/localizador-de-lojas</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Festval Batel</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>4,7</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>5.476</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>R. Cel. Dulcídio, 880 - Batel, Curitiba - PR, 80420-170</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>(41) 3014-1590</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>https://festval.com/</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Mercado Municipal de Curitiba</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>4,7</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>77.570</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Av. Sete de Setembro, 1865 - Centro, Curitiba - PR, 80060-070</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>(41) 3363-3764</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>https://www.mercadomunicipaldecuritiba.com.br/</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Super Muffato Portão</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>4,3</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>22.374</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>R. Eduardo Carlos Pereira, 3605 - Portão, Curitiba - PR, 81020-235</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>(41) 4009-5100</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>http://www.supermuffato.com.br/</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Mercado Vince</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>4,1</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2.769</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>R. André de Barros, 68 - Centro, Curitiba - PR, 80010-080</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>(41) 3018-8589</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Não disponível</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Angeloni Água Verde</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>4,4</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>16.729</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Av. Rep. Argentina, 900 - Água Verde, Curitiba - PR, 80620-010</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>(41) 3312-2300</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>https://www.angeloni.com.br/</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -2788,7 +2468,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="88" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="66" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2826,7 +2506,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Barbearia Garoto Cachoeirinha</t>
+          <t>Stop Studio – Barbearia e Visagismo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2836,29 +2516,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>106</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Av. Bernardo de Vasconcelos, 1193 - Cachoeirinha, Belo Horizonte - MG, 31150-000</t>
+          <t>R. Rio Grande do Norte, 355 - Sala 310 - Santa Efigênia, Belo Horizonte - MG, 30130-130</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>(31) 99328-0816</t>
+          <t>(31) 99147-2866</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://barbeariagaroto.com.br/</t>
+          <t>https://stopstudio.com.br/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Stop Studio – Barbearia e Visagismo</t>
+          <t>All In Barbearia - Álvares Cabral</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2868,29 +2548,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>583</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>R. Rio Grande do Norte, 355 - Sala 310 - Santa Efigênia, Belo Horizonte - MG, 30130-130</t>
+          <t>Av. Álvares Cabral, 1328 - Lourdes, Belo Horizonte - MG, 30170-001</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>(31) 99147-2866</t>
+          <t>(31) 98334-4975</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://stopstudio.com.br/</t>
+          <t>https://www.allinbarbearia.com.br/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>All In Barbearia</t>
+          <t>Barber Town - Belo Horizonte</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2900,29 +2580,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>541</t>
+          <t>260</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Av. Álvares Cabral, 1328 - Lourdes, Belo Horizonte - MG, 30170-001</t>
+          <t>R. Paraíba, 1378 - Loja 113 - Savassi, Belo Horizonte - MG, 30130-148</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>(31) 98334-4975</t>
+          <t>(31) 99119-8729</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.allinbarbearia.com.br/</t>
+          <t>https://api.whatsapp.com/send?phone=5531991198729</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Clube da Barba BH</t>
+          <t>Barbearia Tradicional</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2932,54 +2612,214 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>177</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>R. Gentios, 161 - Loja 2 - Luxemburgo, Belo Horizonte - MG, 30380-490</t>
+          <t>Rua dos Goitacazes, 407 - Centro, Belo Horizonte - MG, 30190-050</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>(31) 97544-9071</t>
+          <t>(31) 99396-9069</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>http://www.clubedabarbabh.com.br/</t>
+          <t>https://bit.ly/3YjAE4q</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Clube da Barba BH</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4,9</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>441</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>R. Gentios, 161 - Loja 2 - Luxemburgo, Belo Horizonte - MG, 30380-490</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>(31) 97544-9071</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>http://www.clubedabarbabh.com.br/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Mens Barbearia</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>5,0</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>689</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Av. Bias Fortes, 851 - Lourdes, Belo Horizonte - MG, 30170-012</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>(31) 3785-8180</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>https://www.mensbarbearia.com.br/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Folk Barbearia</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>5,0</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>605</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Av. Prudente de Morais, 275 - loja 07 - Cidade Jardim, Belo Horizonte - MG, 30350-093</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>(31) 3267-9607</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://folkbarbearia.com.br/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Barbearia Belo Horizonte Luxemburgo</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>4,6</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Rua Guaicuí, 110 - lj 03 - Coracao de Jesus, Belo Horizonte - MG, 30380-342</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>(31) 3021-9791</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://instagram.com/barbeariabelohorizonte?utm_medium=copy_link</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Barbearia do Rapha Savassi</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>5,0</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2.223</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Rua Professor Moraes, 476 - Lj 01 - Funcionários, Belo Horizonte - MG, 30150-370</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>(31) 3055-3007</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>http://www.barbeariadorapha.com.br/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Barbearia La Blade</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>5,0</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>270</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Av. Prudente de Morais, 290 - loja 16 - Cidade Jardim, Belo Horizonte - MG, 30380-002</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Não encontrado</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://sites.appbarber.com.br/labladebarbearia-q26m</t>
         </is>
       </c>
     </row>

</xml_diff>